<commit_message>
Update vendor categories and refresh dashboard outputs
</commit_message>
<xml_diff>
--- a/data/vendor_master.xlsx
+++ b/data/vendor_master.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nvaik11/Documents/projects/OpenClaw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nvaik11/projects/supplier-watchtower/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F201742C-D600-9347-8AA0-732FCE1DF5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D7A22A7-327F-F846-AFCD-9ACFED87F608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="241">
   <si>
     <t>category_id</t>
   </si>
@@ -48,24 +48,6 @@
     <t>High</t>
   </si>
   <si>
-    <t>CAT002</t>
-  </si>
-  <si>
-    <t>Sound Components</t>
-  </si>
-  <si>
-    <t>Speakers microphones receivers and acoustic module suppliers</t>
-  </si>
-  <si>
-    <t>CAT003</t>
-  </si>
-  <si>
-    <t>Packaging</t>
-  </si>
-  <si>
-    <t>Product packaging and retail packaging component suppliers</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
@@ -183,141 +165,12 @@
     <t>Optics and module production</t>
   </si>
   <si>
-    <t>SUP006</t>
-  </si>
-  <si>
-    <t>AAC Technologies</t>
-  </si>
-  <si>
-    <t>https://www.aactechnologies.com</t>
-  </si>
-  <si>
-    <t>Audio component supplier</t>
-  </si>
-  <si>
-    <t>SUP007</t>
-  </si>
-  <si>
-    <t>Goertek</t>
-  </si>
-  <si>
-    <t>https://www.goertek.com</t>
-  </si>
-  <si>
-    <t>Acoustic and wearable electronics supplier</t>
-  </si>
-  <si>
-    <t>SUP008</t>
-  </si>
-  <si>
-    <t>Knowles</t>
-  </si>
-  <si>
     <t>United States</t>
   </si>
   <si>
-    <t>https://www.knowles.com</t>
-  </si>
-  <si>
-    <t>Microphone and precision audio supplier</t>
-  </si>
-  <si>
-    <t>SUP009</t>
-  </si>
-  <si>
-    <t>Foster Electric</t>
-  </si>
-  <si>
-    <t>https://www.foster.co.jp</t>
-  </si>
-  <si>
-    <t>Speaker and acoustic component supplier</t>
-  </si>
-  <si>
-    <t>SUP010</t>
-  </si>
-  <si>
-    <t>MEMSensing Microsystems</t>
-  </si>
-  <si>
-    <t>https://www.memsmicro.com</t>
-  </si>
-  <si>
     <t>Low</t>
   </si>
   <si>
-    <t>MEMS microphone supplier</t>
-  </si>
-  <si>
-    <t>SUP011</t>
-  </si>
-  <si>
-    <t>DS Smith</t>
-  </si>
-  <si>
-    <t>United Kingdom</t>
-  </si>
-  <si>
-    <t>https://www.dssmith.com</t>
-  </si>
-  <si>
-    <t>Sustainable packaging supplier</t>
-  </si>
-  <si>
-    <t>SUP012</t>
-  </si>
-  <si>
-    <t>Smurfit Westrock</t>
-  </si>
-  <si>
-    <t>Ireland</t>
-  </si>
-  <si>
-    <t>https://www.smurfitwestrock.com</t>
-  </si>
-  <si>
-    <t>Global paper and packaging supplier</t>
-  </si>
-  <si>
-    <t>SUP013</t>
-  </si>
-  <si>
-    <t>International Paper</t>
-  </si>
-  <si>
-    <t>https://www.internationalpaper.com</t>
-  </si>
-  <si>
-    <t>Paper based packaging supplier</t>
-  </si>
-  <si>
-    <t>SUP014</t>
-  </si>
-  <si>
-    <t>Oji Holdings</t>
-  </si>
-  <si>
-    <t>https://www.ojiholdings.co.jp</t>
-  </si>
-  <si>
-    <t>Industrial and consumer packaging supplier</t>
-  </si>
-  <si>
-    <t>SUP015</t>
-  </si>
-  <si>
-    <t>Stora Enso</t>
-  </si>
-  <si>
-    <t>Finland</t>
-  </si>
-  <si>
-    <t>https://www.storaenso.com</t>
-  </si>
-  <si>
-    <t>Renewable materials and packaging supplier</t>
-  </si>
-  <si>
     <t>SUP016</t>
   </si>
   <si>
@@ -498,174 +351,9 @@
     <t>Optics and module production site</t>
   </si>
   <si>
-    <t>SITE006</t>
-  </si>
-  <si>
-    <t>AAC Technologies Changzhou Campus</t>
-  </si>
-  <si>
-    <t>Changzhou</t>
-  </si>
-  <si>
     <t>Jiangsu</t>
   </si>
   <si>
-    <t>Changzhou, Jiangsu, China</t>
-  </si>
-  <si>
-    <t>Audio module production site</t>
-  </si>
-  <si>
-    <t>SITE007</t>
-  </si>
-  <si>
-    <t>Goertek Weifang Campus</t>
-  </si>
-  <si>
-    <t>Weifang</t>
-  </si>
-  <si>
-    <t>Shandong</t>
-  </si>
-  <si>
-    <t>Weifang, Shandong, China</t>
-  </si>
-  <si>
-    <t>Large electronics and acoustics site</t>
-  </si>
-  <si>
-    <t>SITE008</t>
-  </si>
-  <si>
-    <t>Knowles Itasca HQ and Engineering</t>
-  </si>
-  <si>
-    <t>Itasca</t>
-  </si>
-  <si>
-    <t>Illinois</t>
-  </si>
-  <si>
-    <t>Itasca, IL, USA</t>
-  </si>
-  <si>
-    <t>Engineering/HQ</t>
-  </si>
-  <si>
-    <t>Public company HQ and engineering presence</t>
-  </si>
-  <si>
-    <t>SITE009</t>
-  </si>
-  <si>
-    <t>Foster Electric Akishima Site</t>
-  </si>
-  <si>
-    <t>Akishima</t>
-  </si>
-  <si>
-    <t>Tokyo</t>
-  </si>
-  <si>
-    <t>Akishima, Tokyo, Japan</t>
-  </si>
-  <si>
-    <t>Audio component manufacturing location</t>
-  </si>
-  <si>
-    <t>SITE010</t>
-  </si>
-  <si>
-    <t>MEMSensing Suzhou Site</t>
-  </si>
-  <si>
-    <t>Suzhou</t>
-  </si>
-  <si>
-    <t>Suzhou, Jiangsu, China</t>
-  </si>
-  <si>
-    <t>MEMS microphone manufacturing site</t>
-  </si>
-  <si>
-    <t>SITE011</t>
-  </si>
-  <si>
-    <t>DS Smith Kemsley Mill</t>
-  </si>
-  <si>
-    <t>Sittingbourne</t>
-  </si>
-  <si>
-    <t>Kent</t>
-  </si>
-  <si>
-    <t>Sittingbourne, Kent, UK</t>
-  </si>
-  <si>
-    <t>Paper and packaging production site</t>
-  </si>
-  <si>
-    <t>SITE012</t>
-  </si>
-  <si>
-    <t>Smurfit Westrock Dublin Office</t>
-  </si>
-  <si>
-    <t>Dublin</t>
-  </si>
-  <si>
-    <t>Dublin, Ireland</t>
-  </si>
-  <si>
-    <t>HQ/Commercial</t>
-  </si>
-  <si>
-    <t>Representative HQ location</t>
-  </si>
-  <si>
-    <t>SITE013</t>
-  </si>
-  <si>
-    <t>International Paper Memphis HQ</t>
-  </si>
-  <si>
-    <t>Memphis</t>
-  </si>
-  <si>
-    <t>Tennessee</t>
-  </si>
-  <si>
-    <t>Memphis, TN, USA</t>
-  </si>
-  <si>
-    <t>Corporate HQ for packaging supplier</t>
-  </si>
-  <si>
-    <t>SITE014</t>
-  </si>
-  <si>
-    <t>Oji Holdings Tokyo HQ</t>
-  </si>
-  <si>
-    <t>Tokyo, Japan</t>
-  </si>
-  <si>
-    <t>Corporate HQ location</t>
-  </si>
-  <si>
-    <t>SITE015</t>
-  </si>
-  <si>
-    <t>Stora Enso Helsinki Office</t>
-  </si>
-  <si>
-    <t>Helsinki</t>
-  </si>
-  <si>
-    <t>Helsinki, Finland</t>
-  </si>
-  <si>
     <t>SITE016</t>
   </si>
   <si>
@@ -751,6 +439,312 @@
   </si>
   <si>
     <t>Amagasaki, Hyogo, Japan</t>
+  </si>
+  <si>
+    <t>CAT006</t>
+  </si>
+  <si>
+    <t>Battery Materials</t>
+  </si>
+  <si>
+    <t>Lithium-ion cells, battery materials, and energy storage suppliers</t>
+  </si>
+  <si>
+    <t>SUP021</t>
+  </si>
+  <si>
+    <t>CATL</t>
+  </si>
+  <si>
+    <t>SUP022</t>
+  </si>
+  <si>
+    <t>LG Energy Solution</t>
+  </si>
+  <si>
+    <t>SUP023</t>
+  </si>
+  <si>
+    <t>Panasonic Energy</t>
+  </si>
+  <si>
+    <t>SUP024</t>
+  </si>
+  <si>
+    <t>Samsung SDI</t>
+  </si>
+  <si>
+    <t>SUP025</t>
+  </si>
+  <si>
+    <t>BYD</t>
+  </si>
+  <si>
+    <t>Chip Modules</t>
+  </si>
+  <si>
+    <t>CAT005</t>
+  </si>
+  <si>
+    <t>Semiconductor packaging testing and chip module suppliers</t>
+  </si>
+  <si>
+    <t>ASE Technology</t>
+  </si>
+  <si>
+    <t>https://www.aseglobal.com</t>
+  </si>
+  <si>
+    <t>Leading OSAT provider</t>
+  </si>
+  <si>
+    <t>Amkor Technology</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>https://www.amkor.com</t>
+  </si>
+  <si>
+    <t>Major semiconductor packaging provider</t>
+  </si>
+  <si>
+    <t>JCET</t>
+  </si>
+  <si>
+    <t>https://www.jcetglobal.com</t>
+  </si>
+  <si>
+    <t>China based OSAT provider</t>
+  </si>
+  <si>
+    <t>Powertech Technology</t>
+  </si>
+  <si>
+    <t>https://www.pti.com.tw</t>
+  </si>
+  <si>
+    <t>Memory packaging specialist</t>
+  </si>
+  <si>
+    <t>Tongfu Microelectronics</t>
+  </si>
+  <si>
+    <t>https://www.tfme.com</t>
+  </si>
+  <si>
+    <t>Chip packaging and testing</t>
+  </si>
+  <si>
+    <t>SUP026</t>
+  </si>
+  <si>
+    <t>https://www.catl.com</t>
+  </si>
+  <si>
+    <t>World largest EV battery supplier</t>
+  </si>
+  <si>
+    <t>SUP027</t>
+  </si>
+  <si>
+    <t>https://www.lgensol.com</t>
+  </si>
+  <si>
+    <t>Global battery manufacturer</t>
+  </si>
+  <si>
+    <t>SUP028</t>
+  </si>
+  <si>
+    <t>https://www.panasonic.com</t>
+  </si>
+  <si>
+    <t>Key Tesla and OEM supplier</t>
+  </si>
+  <si>
+    <t>SUP029</t>
+  </si>
+  <si>
+    <t>https://www.samsungsdi.com</t>
+  </si>
+  <si>
+    <t>Battery and energy storage solutions</t>
+  </si>
+  <si>
+    <t>SUP030</t>
+  </si>
+  <si>
+    <t>https://www.byd.com</t>
+  </si>
+  <si>
+    <t>Integrated EV and battery manufacturer</t>
+  </si>
+  <si>
+    <t>SITE021</t>
+  </si>
+  <si>
+    <t>ASE Kaohsiung Plant</t>
+  </si>
+  <si>
+    <t>Kaohsiung</t>
+  </si>
+  <si>
+    <t>Kaohsiung Taiwan</t>
+  </si>
+  <si>
+    <t>Core semiconductor packaging hub</t>
+  </si>
+  <si>
+    <t>SITE022</t>
+  </si>
+  <si>
+    <t>Amkor Arizona Facility</t>
+  </si>
+  <si>
+    <t>Phoenix</t>
+  </si>
+  <si>
+    <t>Arizona</t>
+  </si>
+  <si>
+    <t>Phoenix Arizona USA</t>
+  </si>
+  <si>
+    <t>US advanced packaging site</t>
+  </si>
+  <si>
+    <t>SITE023</t>
+  </si>
+  <si>
+    <t>JCET Jiangyin Campus</t>
+  </si>
+  <si>
+    <t>Jiangyin</t>
+  </si>
+  <si>
+    <t>Jiangyin Jiangsu China</t>
+  </si>
+  <si>
+    <t>Main China packaging facility</t>
+  </si>
+  <si>
+    <t>SITE024</t>
+  </si>
+  <si>
+    <t>Powertech Hsinchu Plant</t>
+  </si>
+  <si>
+    <t>Hsinchu</t>
+  </si>
+  <si>
+    <t>Hsinchu Taiwan</t>
+  </si>
+  <si>
+    <t>Memory packaging site</t>
+  </si>
+  <si>
+    <t>SITE025</t>
+  </si>
+  <si>
+    <t>Tongfu Nantong Facility</t>
+  </si>
+  <si>
+    <t>Nantong</t>
+  </si>
+  <si>
+    <t>Nantong Jiangsu China</t>
+  </si>
+  <si>
+    <t>Key OSAT production plant</t>
+  </si>
+  <si>
+    <t>SITE026</t>
+  </si>
+  <si>
+    <t>CATL Ningde Facility</t>
+  </si>
+  <si>
+    <t>Ningde</t>
+  </si>
+  <si>
+    <t>Fujian</t>
+  </si>
+  <si>
+    <t>Ningde Fujian China</t>
+  </si>
+  <si>
+    <t>Primary battery production hub</t>
+  </si>
+  <si>
+    <t>SITE027</t>
+  </si>
+  <si>
+    <t>LG Energy Poland Plant</t>
+  </si>
+  <si>
+    <t>Wroclaw</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>Wroclaw Poland</t>
+  </si>
+  <si>
+    <t>EU battery production site</t>
+  </si>
+  <si>
+    <t>SITE028</t>
+  </si>
+  <si>
+    <t>Panasonic Nevada Gigafactory</t>
+  </si>
+  <si>
+    <t>Sparks</t>
+  </si>
+  <si>
+    <t>Nevada</t>
+  </si>
+  <si>
+    <t>Sparks Nevada USA</t>
+  </si>
+  <si>
+    <t>US battery production facility</t>
+  </si>
+  <si>
+    <t>SITE029</t>
+  </si>
+  <si>
+    <t>Samsung SDI Ulsan Plant</t>
+  </si>
+  <si>
+    <t>Ulsan</t>
+  </si>
+  <si>
+    <t>Ulsan South Korea</t>
+  </si>
+  <si>
+    <t>Battery manufacturing site</t>
+  </si>
+  <si>
+    <t>SITE030</t>
+  </si>
+  <si>
+    <t>BYD Shenzhen Campus</t>
+  </si>
+  <si>
+    <t>Shenzhen</t>
+  </si>
+  <si>
+    <t>Guangdong</t>
+  </si>
+  <si>
+    <t>Shenzhen Guangdong China</t>
+  </si>
+  <si>
+    <t>Integrated battery and EV hub</t>
   </si>
 </sst>
 </file>
@@ -938,7 +932,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -953,7 +947,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -966,12 +960,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -981,7 +969,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -994,12 +982,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1009,7 +991,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1022,12 +1004,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1037,7 +1013,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1050,12 +1026,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1065,7 +1035,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1078,12 +1048,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1093,7 +1057,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1106,12 +1070,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1121,7 +1079,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1134,12 +1092,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1149,7 +1101,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1162,12 +1114,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1177,7 +1123,7 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1190,124 +1136,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1325,254 +1153,6 @@
           <bgColor theme="2"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1675,10 +1255,21 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1695,6 +1286,409 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1719,53 +1713,53 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CategoriesTable" displayName="CategoriesTable" ref="A1:D5" headerRowDxfId="25" dataDxfId="32" totalsRowDxfId="24" headerRowBorderDxfId="30" tableBorderDxfId="31">
-  <autoFilter ref="A1:D5" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CategoriesTable" displayName="CategoriesTable" ref="A1:D8" headerRowDxfId="18" dataDxfId="16" totalsRowDxfId="14" headerRowBorderDxfId="17" tableBorderDxfId="15">
+  <autoFilter ref="A1:D8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="category_id" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="category_name" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="category_description" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="strategic_priority" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="category_id" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="category_name" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="category_description" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="strategic_priority" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="SuppliersTable" displayName="SuppliersTable" ref="A1:I21" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="SuppliersTable" displayName="SuppliersTable" ref="A1:I21" dataDxfId="9">
   <autoFilter ref="A1:I21" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="supplier_id" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="supplier_name" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="category_id" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="hq_country" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="public_company" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="website" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="monitoring_priority" dataDxfId="17"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="status" dataDxfId="16"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="notes" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="supplier_id" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="supplier_name" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="category_id" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="hq_country" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="public_company" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="website" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="monitoring_priority" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="status" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="SitesTable" displayName="SitesTable" ref="A1:M21" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="SitesTable" displayName="SitesTable" ref="A1:M21" dataDxfId="32">
   <autoFilter ref="A1:M21" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="site_id" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="supplier_id" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="site_name" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="city" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="state_region" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="country" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="address" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="site_type" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="latitude" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="longitude" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="primary_site" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="is_monitored" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="notes" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="site_id" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="supplier_id" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="site_name" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="city" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="state_region" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="country" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="address" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="site_type" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="latitude" dataDxfId="23"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="longitude" dataDxfId="22"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="primary_site" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="is_monitored" dataDxfId="20"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="notes" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2056,7 +2050,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -2094,46 +2088,64 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="B3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>13</v>
+        <v>153</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>154</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="A5" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>7</v>
       </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="4"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="4"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2160,611 +2172,611 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>7</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="H3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11" s="5" t="s">
         <v>70</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>75</v>
+        <v>142</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>76</v>
+        <v>155</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>11</v>
+        <v>153</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>79</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>80</v>
+        <v>144</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>11</v>
+        <v>153</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>82</v>
+        <v>159</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>83</v>
+        <v>160</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>84</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>85</v>
+        <v>146</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>86</v>
+        <v>162</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>11</v>
+        <v>153</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>87</v>
+        <v>163</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>88</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>89</v>
+        <v>148</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>90</v>
+        <v>165</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>11</v>
+        <v>153</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="E15" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>95</v>
-      </c>
       <c r="E16" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>96</v>
+        <v>169</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>97</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>98</v>
+        <v>171</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>99</v>
+        <v>143</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>15</v>
+        <v>139</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>100</v>
+        <v>172</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>7</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>101</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>102</v>
+        <v>174</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>15</v>
+        <v>139</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>104</v>
+        <v>175</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>7</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>105</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>106</v>
+        <v>177</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>107</v>
+        <v>147</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>15</v>
+        <v>139</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>108</v>
+        <v>38</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>109</v>
+        <v>178</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>110</v>
+        <v>25</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>111</v>
+        <v>179</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>15</v>
+        <v>139</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>44</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>114</v>
+        <v>181</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>115</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>116</v>
+        <v>183</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>15</v>
+        <v>139</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>118</v>
+        <v>184</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>119</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2795,773 +2807,771 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>120</v>
+        <v>71</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>121</v>
+        <v>72</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>122</v>
+        <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>123</v>
+        <v>74</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>124</v>
+        <v>75</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>125</v>
+        <v>76</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>126</v>
+        <v>77</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>127</v>
+        <v>78</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>128</v>
+        <v>79</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>129</v>
+        <v>80</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>130</v>
+        <v>81</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>132</v>
+        <v>83</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>133</v>
+        <v>84</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>134</v>
+        <v>85</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>136</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>137</v>
+        <v>88</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>138</v>
+        <v>89</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>140</v>
+        <v>91</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>141</v>
+        <v>92</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>142</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>143</v>
+        <v>94</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>144</v>
+        <v>95</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>133</v>
+        <v>84</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>134</v>
+        <v>85</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>145</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>146</v>
+        <v>97</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>150</v>
+        <v>101</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>151</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>152</v>
+        <v>103</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>153</v>
+        <v>104</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>155</v>
+        <v>106</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>156</v>
+        <v>107</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>157</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>158</v>
+        <v>110</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>159</v>
+        <v>111</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>160</v>
+        <v>112</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>161</v>
+        <v>113</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>162</v>
+        <v>114</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
       <c r="K7" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>163</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>164</v>
+        <v>116</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>165</v>
+        <v>117</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>166</v>
+        <v>118</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>167</v>
+        <v>119</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>169</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>170</v>
+        <v>122</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>171</v>
+        <v>123</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>172</v>
+        <v>124</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>173</v>
+        <v>125</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>174</v>
+        <v>126</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>175</v>
+        <v>86</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>176</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>178</v>
+        <v>129</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>179</v>
+        <v>130</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>180</v>
+        <v>131</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>181</v>
+        <v>132</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>182</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>183</v>
+        <v>134</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>184</v>
+        <v>135</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>185</v>
+        <v>136</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>186</v>
+        <v>138</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>187</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="E12" s="5"/>
+      <c r="F12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>192</v>
-      </c>
       <c r="H12" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="F13" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>197</v>
-      </c>
       <c r="H13" s="5" t="s">
-        <v>198</v>
+        <v>86</v>
       </c>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>204</v>
-      </c>
       <c r="H14" s="5" t="s">
-        <v>198</v>
+        <v>86</v>
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>89</v>
+        <v>148</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>198</v>
+        <v>86</v>
       </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>213</v>
-      </c>
       <c r="H16" s="5" t="s">
-        <v>198</v>
+        <v>86</v>
       </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
       <c r="K16" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="F17" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>218</v>
-      </c>
       <c r="H17" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C18" s="5" t="s">
+      <c r="E18" s="5"/>
+      <c r="F18" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="G18" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>224</v>
-      </c>
       <c r="H18" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="F19" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>230</v>
-      </c>
       <c r="H19" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>235</v>
-      </c>
+      <c r="E20" s="5"/>
       <c r="F20" s="5" t="s">
         <v>44</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
       <c r="K20" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M20" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="F21" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="L20" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M20" s="5" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C21" s="5" t="s">
+      <c r="G21" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="H21" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="L21" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M21" s="8" t="s">
         <v>240</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="L21" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M21" s="5" t="s">
-        <v>237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>